<commit_message>
Here i am writting test cases for report generation.....
</commit_message>
<xml_diff>
--- a/testdata/data.xlsx
+++ b/testdata/data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pavan\OneDrive\Desktop\testdata\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ASUS\PycharmProjects\PWPython\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CA45082-25B2-4B3B-8413-73A82F09A22F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8715CF20-0CD3-4FBB-B2F8-3B647EA6835D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="16354" yWindow="-103" windowWidth="33120" windowHeight="18000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -445,14 +445,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="39.54296875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.1796875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.90625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="39.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.21875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="21" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" ht="42" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -463,7 +463,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="21" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" ht="42" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
@@ -474,7 +474,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="21" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" ht="21" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>6</v>
       </c>
@@ -485,7 +485,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="21" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" ht="21" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>8</v>
       </c>
@@ -496,7 +496,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="21" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" ht="21" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
         <v>11</v>
       </c>

</xml_diff>